<commit_message>
actualizaciónd de la documentación con iteraicón 5
</commit_message>
<xml_diff>
--- a/docs/seguimiento/commits_por_iteracion.xlsx
+++ b/docs/seguimiento/commits_por_iteracion.xlsx
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D92"/>
+  <dimension ref="A1:D96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2525,6 +2525,94 @@
         </is>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" s="12" t="inlineStr">
+        <is>
+          <t>Ignacio</t>
+        </is>
+      </c>
+      <c r="B93" s="12" t="inlineStr">
+        <is>
+          <t>Iteracion 5</t>
+        </is>
+      </c>
+      <c r="C93" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D93" s="12" t="inlineStr">
+        <is>
+          <t>Dueno: permisos Eventos + filtro por unidad en GetEventos (follow-up RF-15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="12" t="inlineStr">
+        <is>
+          <t>Ignacio</t>
+        </is>
+      </c>
+      <c r="B94" s="12" t="inlineStr">
+        <is>
+          <t>Iteracion 5</t>
+        </is>
+      </c>
+      <c r="C94" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D94" s="12" t="inlineStr">
+        <is>
+          <t>Notificaciones: fix take del listado del portal (Math.Clamp)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="12" t="inlineStr">
+        <is>
+          <t>Ignacio</t>
+        </is>
+      </c>
+      <c r="B95" s="12" t="inlineStr">
+        <is>
+          <t>Iteracion 5</t>
+        </is>
+      </c>
+      <c r="C95" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D95" s="12" t="inlineStr">
+        <is>
+          <t>MFA: CI workflow manual para cargar claves en Container App</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="12" t="inlineStr">
+        <is>
+          <t>Sebastian</t>
+        </is>
+      </c>
+      <c r="B96" s="12" t="inlineStr">
+        <is>
+          <t>Iteracion 5</t>
+        </is>
+      </c>
+      <c r="C96" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="D96" s="12" t="inlineStr">
+        <is>
+          <t>Docs: mejoras de documentacion</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D92"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>